<commit_message>
testdata: add exemplar anonymouse xlsx files
</commit_message>
<xml_diff>
--- a/testdata/enthuse_bad_first_sheet.xlsx
+++ b/testdata/enthuse_bad_first_sheet.xlsx
@@ -21,11 +21,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t xml:space="preserve">Some summary data</t>
   </si>
   <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Payment ID</t>
   </si>
   <si>
@@ -89,7 +98,13 @@
     <t xml:space="preserve">Fundraising Page ID</t>
   </si>
   <si>
-    <t xml:space="preserve">py_2SZANObc13bvgL6ja</t>
+    <t xml:space="preserve">Fundraising &amp; Donations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">py_abcdef2SZANN6oA613bvgL6ja</t>
   </si>
   <si>
     <t xml:space="preserve">xxx</t>
@@ -110,13 +125,13 @@
     <t xml:space="preserve">Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">py_2Saionabc0yICk10Qb</t>
+    <t xml:space="preserve">py_abcdef2Saion6OM60yICk10Qb</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">ch_2Sbdefg26OMOHD7c</t>
+    <t xml:space="preserve">ch_abcdef2Sb8q26OA60KAgOHD7c</t>
   </si>
   <si>
     <t xml:space="preserve">Anonymous</t>
@@ -129,8 +144,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -209,7 +225,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -219,6 +235,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -487,19 +507,19 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="n">
         <f aca="false">'enthusePayout-paid-2025-12-15_e'!L2</f>
-        <v>4.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="n">
         <f aca="false">'enthusePayout-paid-2025-12-15_e'!L3</f>
-        <v>9.38</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="n">
         <f aca="false">'enthusePayout-paid-2025-12-15_e'!L4</f>
-        <v>9.38</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -521,254 +541,272 @@
   <dimension ref="A1:X4"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="22.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>21</v>
+      <c r="V1" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>8157399</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="A2" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="B2" s="3" t="n">
+        <v>45965.0165046296</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="D2" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>9157399</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="L2" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="M2" s="0" t="n">
         <v>0.4</v>
       </c>
-      <c r="K2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="1" t="n">
+      <c r="N2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="0" t="n">
         <v>4.6</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="0" t="n">
         <v>123457</v>
       </c>
-      <c r="S2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" s="1" t="n">
+      <c r="V2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>45965.8389236111</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>9157398</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>8157398</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="1" t="n">
+      <c r="J3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="M3" s="0" t="n">
         <v>0.62</v>
       </c>
-      <c r="K3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="1" t="n">
+      <c r="N3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="0" t="n">
         <v>9.38</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="N3" s="1" t="n">
+      <c r="P3" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q3" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="O3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P3" s="1" t="n">
+      <c r="R3" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="0" t="n">
         <v>123456</v>
       </c>
-      <c r="S3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="1" t="n">
+      <c r="V3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>45966.9965856482</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>9848690</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>6848690</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="L4" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" s="0" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="N4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="0" t="n">
+        <v>9.38</v>
+      </c>
+      <c r="P4" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q4" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="R4" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>9.38</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="N4" s="1" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" s="1" t="n">
+      <c r="S4" s="0" t="n">
         <v>123455</v>
       </c>
-      <c r="S4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="1" t="n">
+      <c r="V4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="0" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" display="email@test.com"/>
-    <hyperlink ref="G3" r:id="rId2" display="email@test.com"/>
+    <hyperlink ref="J2" r:id="rId1" display="email@test.com"/>
+    <hyperlink ref="J3" r:id="rId2" display="email@test.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
testdata: update example excel file
</commit_message>
<xml_diff>
--- a/testdata/enthuse_bad_first_sheet.xlsx
+++ b/testdata/enthuse_bad_first_sheet.xlsx
@@ -238,7 +238,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -539,267 +539,269 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:X4"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="22.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="28.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="5" style="0" width="8.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="T1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="0" t="s">
+      <c r="U1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="0" t="s">
+      <c r="V1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="W1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="0" t="s">
+      <c r="X1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>45965.0165046296</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="2" t="n">
         <v>9157399</v>
       </c>
-      <c r="F2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="0" t="s">
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="J2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="0" t="n">
+      <c r="L2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M2" s="0" t="n">
+      <c r="M2" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="N2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="0" t="n">
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="n">
         <v>4.6</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="P2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="0" t="s">
+      <c r="Q2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="S2" s="0" t="n">
+      <c r="S2" s="2" t="n">
         <v>123457</v>
       </c>
-      <c r="V2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" s="0" t="n">
+      <c r="V2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>45965.8389236111</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="2" t="n">
         <v>9157398</v>
       </c>
-      <c r="F3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="0" t="n">
+      <c r="L3" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M3" s="0" t="n">
+      <c r="M3" s="2" t="n">
         <v>0.62</v>
       </c>
-      <c r="N3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="0" t="n">
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
         <v>9.38</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="P3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q3" s="0" t="n">
+      <c r="Q3" s="2" t="n">
         <v>2.5</v>
       </c>
-      <c r="R3" s="0" t="s">
+      <c r="R3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="0" t="n">
+      <c r="S3" s="2" t="n">
         <v>123456</v>
       </c>
-      <c r="V3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="0" t="n">
+      <c r="V3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>45966.9965856482</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="2" t="n">
         <v>9848690</v>
       </c>
-      <c r="F4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="0" t="s">
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L4" s="0" t="n">
+      <c r="L4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M4" s="0" t="n">
+      <c r="M4" s="2" t="n">
         <v>0.62</v>
       </c>
-      <c r="N4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="0" t="n">
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="n">
         <v>9.38</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="P4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q4" s="0" t="n">
+      <c r="Q4" s="2" t="n">
         <v>2.5</v>
       </c>
-      <c r="R4" s="0" t="s">
+      <c r="R4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="S4" s="0" t="n">
+      <c r="S4" s="2" t="n">
         <v>123455</v>
       </c>
-      <c r="V4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="0" t="n">
+      <c r="V4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>